<commit_message>
community check unique community name
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/CommunityDatabase.xlsx
+++ b/App/CLI-backend/databases/CommunityDatabase.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Name</t>
   </si>
@@ -24,6 +24,18 @@
   </si>
   <si>
     <t>Community creator</t>
+  </si>
+  <si>
+    <t>r/sfeu la bani</t>
+  </si>
+  <si>
+    <t>Science</t>
+  </si>
+  <si>
+    <t>sa</t>
+  </si>
+  <si>
+    <t>admin</t>
   </si>
 </sst>
 </file>
@@ -68,13 +80,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="5.70703125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="5.2578125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.1015625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="16.5390625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="11.53515625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="6.95703125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="10.1015625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="16.5390625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -91,6 +103,20 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
user and community duplicate logic is separated from excelread
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/CommunityDatabase.xlsx
+++ b/App/CLI-backend/databases/CommunityDatabase.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>Name</t>
   </si>
@@ -32,12 +32,31 @@
   </si>
   <si>
     <t>Community creator</t>
+  </si>
+  <si>
+    <t>r/muie</t>
+  </si>
+  <si>
+    <t>Science</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>r/salut</t>
+  </si>
+  <si>
+    <t>sa</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -403,27 +422,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="5.91015625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="7.3125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="9.91015625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="16.1015625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
deleted communities are also deleted from excel
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/CommunityDatabase.xlsx
+++ b/App/CLI-backend/databases/CommunityDatabase.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\serba\AppData\Roaming\SPB_Data\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>Name</t>
   </si>
@@ -32,12 +32,40 @@
   </si>
   <si>
     <t>Community creator</t>
+  </si>
+  <si>
+    <t>r/muie</t>
+  </si>
+  <si>
+    <t>Science</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>r/e</t>
+  </si>
+  <si>
+    <t>sa</t>
+  </si>
+  <si>
+    <t>r/ce zici</t>
+  </si>
+  <si>
+    <t>Art</t>
+  </si>
+  <si>
+    <t>mm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -406,23 +434,23 @@
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="7.0078125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="7.3125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="9.91015625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="16.1015625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Finished both post and comment databases
</commit_message>
<xml_diff>
--- a/App/CLI-backend/databases/CommunityDatabase.xlsx
+++ b/App/CLI-backend/databases/CommunityDatabase.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\serba\AppData\Roaming\SPB_Data\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\ZTH-Team-Deltaspace\App\CLI-backend\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58640FE0-73F2-4ED1-93C0-578BD4F6480B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CA496A-DFAD-4CC4-A94F-A2BDC540AEBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1896" yWindow="3288" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet0" sheetId="1" r:id="rId1"/>
@@ -20,20 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Topic</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Community creator</t>
-  </si>
-</sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -403,30 +390,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>